<commit_message>
Build formula-driven Excel models: upload, choose models, download one workbook
- New Build Excel Model page: upload statements, tick the models to include
  (or select all), download a single workbook
- excel.js builds real Excel models with ExcelJS (loaded on demand): Cover,
  Historicals and one sheet per model, with live formulas, blue inputs,
  green links to Historicals and banker-style formatting
- A built-in formula evaluator stores calculated values, so files open with
  correct numbers in any viewer; Excel also recalculates on load
- Model and Feasibility 'Download Excel' buttons now produce the same
  formula-driven workbooks; the old value-only export is removed
- Monte Carlo and Feasibility calculations shared between app and workbook
- Regenerated sample workbooks, plus full-financial-model.xlsx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8KFsQTUuD7H1QVgxuxefc
</commit_message>
<xml_diff>
--- a/samples/models/powerbi-dataset.xlsx
+++ b/samples/models/powerbi-dataset.xlsx
@@ -420,7 +420,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B2">
         <v>2020</v>
@@ -437,7 +437,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B3">
         <v>2021</v>
@@ -454,7 +454,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B4">
         <v>2022</v>
@@ -471,7 +471,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B5">
         <v>2023</v>
@@ -488,7 +488,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B6">
         <v>2024</v>
@@ -505,7 +505,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B7">
         <v>2020</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B8">
         <v>2021</v>
@@ -539,7 +539,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B9">
         <v>2022</v>
@@ -556,7 +556,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B10">
         <v>2023</v>
@@ -573,7 +573,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B11">
         <v>2024</v>
@@ -590,7 +590,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B12">
         <v>2020</v>
@@ -607,7 +607,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B13">
         <v>2021</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B14">
         <v>2022</v>
@@ -641,7 +641,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B15">
         <v>2023</v>
@@ -658,7 +658,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B16">
         <v>2024</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B17">
         <v>2020</v>
@@ -692,7 +692,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B18">
         <v>2021</v>
@@ -709,7 +709,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B19">
         <v>2022</v>
@@ -726,7 +726,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B20">
         <v>2023</v>
@@ -743,7 +743,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B21">
         <v>2024</v>
@@ -760,7 +760,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B22">
         <v>2020</v>
@@ -777,7 +777,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B23">
         <v>2021</v>
@@ -794,7 +794,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B24">
         <v>2022</v>
@@ -811,7 +811,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B25">
         <v>2023</v>
@@ -828,7 +828,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B26">
         <v>2024</v>
@@ -845,7 +845,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B27">
         <v>2020</v>
@@ -862,7 +862,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B28">
         <v>2021</v>
@@ -879,7 +879,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B29">
         <v>2022</v>
@@ -896,7 +896,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B30">
         <v>2023</v>
@@ -913,7 +913,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B31">
         <v>2024</v>
@@ -930,7 +930,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B32">
         <v>2020</v>
@@ -947,7 +947,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B33">
         <v>2021</v>
@@ -964,7 +964,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B34">
         <v>2022</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B35">
         <v>2023</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B36">
         <v>2024</v>
@@ -1015,7 +1015,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B37">
         <v>2020</v>
@@ -1032,7 +1032,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B38">
         <v>2021</v>
@@ -1049,7 +1049,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B39">
         <v>2022</v>
@@ -1066,7 +1066,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B40">
         <v>2023</v>
@@ -1083,7 +1083,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B41">
         <v>2024</v>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B42">
         <v>2020</v>
@@ -1117,7 +1117,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B43">
         <v>2021</v>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B44">
         <v>2022</v>
@@ -1151,7 +1151,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B45">
         <v>2023</v>
@@ -1168,7 +1168,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B46">
         <v>2024</v>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B47">
         <v>2020</v>
@@ -1202,7 +1202,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B48">
         <v>2021</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B49">
         <v>2022</v>
@@ -1236,7 +1236,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B50">
         <v>2023</v>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B51">
         <v>2024</v>
@@ -1270,7 +1270,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B52">
         <v>2020</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B53">
         <v>2021</v>
@@ -1304,7 +1304,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B54">
         <v>2022</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B55">
         <v>2023</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B56">
         <v>2024</v>
@@ -1355,7 +1355,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B57">
         <v>2020</v>
@@ -1372,7 +1372,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B58">
         <v>2021</v>
@@ -1389,7 +1389,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B59">
         <v>2022</v>
@@ -1406,7 +1406,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B60">
         <v>2023</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B61">
         <v>2024</v>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B62">
         <v>2020</v>
@@ -1457,7 +1457,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B63">
         <v>2021</v>
@@ -1474,7 +1474,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B64">
         <v>2022</v>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B65">
         <v>2023</v>
@@ -1508,7 +1508,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B66">
         <v>2024</v>
@@ -1525,7 +1525,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B67">
         <v>2020</v>
@@ -1542,7 +1542,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B68">
         <v>2021</v>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B69">
         <v>2022</v>
@@ -1576,7 +1576,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B70">
         <v>2023</v>
@@ -1593,7 +1593,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B71">
         <v>2024</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B72">
         <v>2020</v>
@@ -1627,7 +1627,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B73">
         <v>2021</v>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B74">
         <v>2022</v>
@@ -1661,7 +1661,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B75">
         <v>2023</v>
@@ -1678,7 +1678,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B76">
         <v>2024</v>
@@ -1695,7 +1695,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B77">
         <v>2020</v>
@@ -1712,7 +1712,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B78">
         <v>2021</v>
@@ -1729,7 +1729,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B79">
         <v>2022</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B80">
         <v>2023</v>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B81">
         <v>2024</v>
@@ -1780,7 +1780,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B82">
         <v>2020</v>
@@ -1797,7 +1797,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B83">
         <v>2021</v>
@@ -1814,7 +1814,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B84">
         <v>2022</v>
@@ -1831,7 +1831,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B85">
         <v>2023</v>
@@ -1848,7 +1848,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B86">
         <v>2024</v>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B87">
         <v>2020</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B88">
         <v>2021</v>
@@ -1899,7 +1899,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B89">
         <v>2022</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B90">
         <v>2023</v>
@@ -1933,7 +1933,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B91">
         <v>2024</v>
@@ -1978,7 +1978,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B2">
         <v>2020</v>
@@ -1995,7 +1995,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B3">
         <v>2020</v>
@@ -2012,7 +2012,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B4">
         <v>2020</v>
@@ -2029,7 +2029,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B5">
         <v>2020</v>
@@ -2046,7 +2046,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B6">
         <v>2020</v>
@@ -2063,7 +2063,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B7">
         <v>2020</v>
@@ -2080,7 +2080,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B8">
         <v>2020</v>
@@ -2097,7 +2097,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B9">
         <v>2020</v>
@@ -2114,7 +2114,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B10">
         <v>2020</v>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B11">
         <v>2020</v>
@@ -2148,7 +2148,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B12">
         <v>2021</v>
@@ -2165,7 +2165,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B13">
         <v>2021</v>
@@ -2182,7 +2182,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B14">
         <v>2021</v>
@@ -2199,7 +2199,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B15">
         <v>2021</v>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B16">
         <v>2021</v>
@@ -2233,7 +2233,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B17">
         <v>2021</v>
@@ -2250,7 +2250,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B18">
         <v>2021</v>
@@ -2267,7 +2267,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B19">
         <v>2021</v>
@@ -2284,7 +2284,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B20">
         <v>2021</v>
@@ -2301,7 +2301,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B21">
         <v>2021</v>
@@ -2318,7 +2318,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B22">
         <v>2021</v>
@@ -2335,7 +2335,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B23">
         <v>2022</v>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B24">
         <v>2022</v>
@@ -2369,7 +2369,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B25">
         <v>2022</v>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B26">
         <v>2022</v>
@@ -2403,7 +2403,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B27">
         <v>2022</v>
@@ -2420,7 +2420,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B28">
         <v>2022</v>
@@ -2437,7 +2437,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B29">
         <v>2022</v>
@@ -2454,7 +2454,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B30">
         <v>2022</v>
@@ -2471,7 +2471,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B31">
         <v>2022</v>
@@ -2488,7 +2488,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B32">
         <v>2022</v>
@@ -2505,7 +2505,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B33">
         <v>2022</v>
@@ -2522,7 +2522,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B34">
         <v>2023</v>
@@ -2539,7 +2539,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B35">
         <v>2023</v>
@@ -2556,7 +2556,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B36">
         <v>2023</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B37">
         <v>2023</v>
@@ -2590,7 +2590,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B38">
         <v>2023</v>
@@ -2607,7 +2607,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B39">
         <v>2023</v>
@@ -2624,7 +2624,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B40">
         <v>2023</v>
@@ -2641,7 +2641,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B41">
         <v>2023</v>
@@ -2658,7 +2658,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B42">
         <v>2023</v>
@@ -2675,7 +2675,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B43">
         <v>2023</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B44">
         <v>2023</v>
@@ -2709,7 +2709,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B45">
         <v>2024</v>
@@ -2726,7 +2726,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B46">
         <v>2024</v>
@@ -2743,7 +2743,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B47">
         <v>2024</v>
@@ -2760,7 +2760,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B48">
         <v>2024</v>
@@ -2777,7 +2777,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B49">
         <v>2024</v>
@@ -2794,7 +2794,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B50">
         <v>2024</v>
@@ -2811,7 +2811,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B51">
         <v>2024</v>
@@ -2828,7 +2828,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B52">
         <v>2024</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B53">
         <v>2024</v>
@@ -2862,7 +2862,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B54">
         <v>2024</v>
@@ -2879,7 +2879,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Aurora Retail Co. (sample)</v>
+        <v>Aurora Retail Co.</v>
       </c>
       <c r="B55">
         <v>2024</v>

</xml_diff>